<commit_message>
Subimos cambios para generar respaldo de cambio de equipo
</commit_message>
<xml_diff>
--- a/MazdaMX2/Dealers.xlsx
+++ b/MazdaMX2/Dealers.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mvelasc2\source\repos\MazdaMX2\MazdaMX2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FC1A355-7D33-43BA-8E28-781C6A5CFE37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{675549AD-CE16-4874-9755-C2AD9D21E7AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15675" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-118" yWindow="-118" windowWidth="25370" windowHeight="13667" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="2" r:id="rId1"/>
@@ -244,9 +244,6 @@
     <t>137</t>
   </si>
   <si>
-    <t>495,900</t>
-  </si>
-  <si>
     <t>Signature MHEV</t>
   </si>
   <si>
@@ -259,9 +256,6 @@
     <t>3.3L</t>
   </si>
   <si>
-    <t>mazda-cx-70-lateral-inclinado-v2</t>
-  </si>
-  <si>
     <t>MAZDA CX-70</t>
   </si>
   <si>
@@ -274,24 +268,6 @@
     <t>332</t>
   </si>
   <si>
-    <t>453,900</t>
-  </si>
-  <si>
-    <t>563,900</t>
-  </si>
-  <si>
-    <t>815,900</t>
-  </si>
-  <si>
-    <t>436,900</t>
-  </si>
-  <si>
-    <t>466,900</t>
-  </si>
-  <si>
-    <t>512,900</t>
-  </si>
-  <si>
     <t>552,900</t>
   </si>
   <si>
@@ -301,63 +277,12 @@
     <t>mazda-cx-50-flydown-v2</t>
   </si>
   <si>
-    <t>386,900</t>
-  </si>
-  <si>
-    <t>416,900</t>
-  </si>
-  <si>
-    <t>mazda-mazda2-sedan-rojo-perfil-v1</t>
-  </si>
-  <si>
-    <t>automovil-mazda2-hatchback-rojo-costado</t>
-  </si>
-  <si>
     <t>mazda-mexico-cx-3-flydown-perfil-v1</t>
   </si>
   <si>
-    <t>548,900</t>
-  </si>
-  <si>
-    <t>608,900</t>
-  </si>
-  <si>
-    <t>678,900</t>
-  </si>
-  <si>
     <t>mazda3-sedan-flydown-perfil-v2</t>
   </si>
   <si>
-    <t>397,900</t>
-  </si>
-  <si>
-    <t>437,900</t>
-  </si>
-  <si>
-    <t>477,900</t>
-  </si>
-  <si>
-    <t>547,900</t>
-  </si>
-  <si>
-    <t>958,000</t>
-  </si>
-  <si>
-    <t>mazda-cx-90-flydown-rojo-artesano-inclinado-v1.png</t>
-  </si>
-  <si>
-    <t>1,058,000</t>
-  </si>
-  <si>
-    <t>300,900</t>
-  </si>
-  <si>
-    <t>330,900</t>
-  </si>
-  <si>
-    <t>370,900</t>
-  </si>
-  <si>
     <t>398,900</t>
   </si>
   <si>
@@ -388,13 +313,88 @@
     <t>MAZDA BT-50</t>
   </si>
   <si>
-    <t>829,900</t>
-  </si>
-  <si>
     <t>3.0L</t>
   </si>
   <si>
     <t>mazda-bt-50-roja-flydown-inclinado-v2</t>
+  </si>
+  <si>
+    <t>403,900</t>
+  </si>
+  <si>
+    <t>442,900</t>
+  </si>
+  <si>
+    <t>482,900</t>
+  </si>
+  <si>
+    <t>458,900</t>
+  </si>
+  <si>
+    <t>498,900</t>
+  </si>
+  <si>
+    <t>568,900</t>
+  </si>
+  <si>
+    <t>441,900</t>
+  </si>
+  <si>
+    <t>471,900</t>
+  </si>
+  <si>
+    <t>517,900</t>
+  </si>
+  <si>
+    <t>557,900</t>
+  </si>
+  <si>
+    <t>391,900</t>
+  </si>
+  <si>
+    <t>421,900</t>
+  </si>
+  <si>
+    <t>551,900</t>
+  </si>
+  <si>
+    <t>611,900</t>
+  </si>
+  <si>
+    <t>681,900</t>
+  </si>
+  <si>
+    <t>818,900</t>
+  </si>
+  <si>
+    <t>961,000</t>
+  </si>
+  <si>
+    <t>1,061,000</t>
+  </si>
+  <si>
+    <t>mazda-cx-70-racks-flydown-inclinado-v1</t>
+  </si>
+  <si>
+    <t>mazda-cx-90-flydown-rojo-artesano-inclinado-v1</t>
+  </si>
+  <si>
+    <t>799,900</t>
+  </si>
+  <si>
+    <t>mazda2-sedan-rojo-auto-perfil-v1</t>
+  </si>
+  <si>
+    <t>mazda2-hatchback-flydown-perfil-v1</t>
+  </si>
+  <si>
+    <t>301,900</t>
+  </si>
+  <si>
+    <t>331,900</t>
+  </si>
+  <si>
+    <t>371,900</t>
   </si>
 </sst>
 </file>
@@ -718,30 +718,30 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AJ15"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.75" defaultRowHeight="15.75"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.77734375" defaultRowHeight="15.75"/>
   <cols>
-    <col min="1" max="1" width="12.75" customWidth="1"/>
-    <col min="2" max="2" width="30.375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.75" customWidth="1"/>
-    <col min="4" max="4" width="12.125" customWidth="1"/>
-    <col min="5" max="5" width="10.75" customWidth="1"/>
+    <col min="1" max="1" width="12.77734375" customWidth="1"/>
+    <col min="2" max="2" width="30.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.77734375" customWidth="1"/>
+    <col min="4" max="4" width="12.109375" customWidth="1"/>
+    <col min="5" max="5" width="10.77734375" customWidth="1"/>
     <col min="6" max="6" width="8" customWidth="1"/>
-    <col min="7" max="7" width="13.25" customWidth="1"/>
+    <col min="7" max="7" width="13.21875" customWidth="1"/>
     <col min="8" max="8" width="9" style="1"/>
     <col min="9" max="9" width="4" style="1" customWidth="1"/>
-    <col min="10" max="10" width="8.75" style="1" customWidth="1"/>
-    <col min="11" max="11" width="9.25" style="1" customWidth="1"/>
-    <col min="12" max="12" width="13.25" customWidth="1"/>
+    <col min="10" max="10" width="8.77734375" style="1" customWidth="1"/>
+    <col min="11" max="11" width="9.21875" style="1" customWidth="1"/>
+    <col min="12" max="12" width="13.21875" customWidth="1"/>
     <col min="13" max="13" width="9" style="1"/>
-    <col min="14" max="15" width="8.75" style="1"/>
-    <col min="16" max="16" width="9.25" style="1" customWidth="1"/>
-    <col min="17" max="17" width="13.75" customWidth="1"/>
+    <col min="14" max="15" width="8.77734375" style="1"/>
+    <col min="16" max="16" width="9.21875" style="1" customWidth="1"/>
+    <col min="17" max="17" width="13.77734375" customWidth="1"/>
     <col min="18" max="18" width="9" style="1"/>
-    <col min="19" max="21" width="8.75" style="1"/>
-    <col min="22" max="22" width="13.875" customWidth="1"/>
-    <col min="25" max="25" width="8.75" customWidth="1"/>
-    <col min="27" max="27" width="10.125" customWidth="1"/>
-    <col min="32" max="32" width="13.875" customWidth="1"/>
+    <col min="19" max="21" width="8.77734375" style="1"/>
+    <col min="22" max="22" width="13.88671875" customWidth="1"/>
+    <col min="25" max="25" width="8.77734375" customWidth="1"/>
+    <col min="27" max="27" width="10.109375" customWidth="1"/>
+    <col min="32" max="32" width="13.88671875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:36">
@@ -859,7 +859,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>95</v>
+        <v>120</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>64</v>
@@ -871,13 +871,13 @@
         <v>36</v>
       </c>
       <c r="F2">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="G2" t="s">
         <v>37</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>109</v>
+        <v>122</v>
       </c>
       <c r="I2" s="1" t="s">
         <v>38</v>
@@ -892,7 +892,7 @@
         <v>41</v>
       </c>
       <c r="M2" s="3" t="s">
-        <v>110</v>
+        <v>123</v>
       </c>
       <c r="N2" s="1" t="s">
         <v>38</v>
@@ -907,7 +907,7 @@
         <v>49</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>111</v>
+        <v>124</v>
       </c>
       <c r="S2" s="3" t="s">
         <v>38</v>
@@ -922,7 +922,7 @@
         <v>50</v>
       </c>
       <c r="W2" s="3" t="s">
-        <v>112</v>
+        <v>87</v>
       </c>
       <c r="X2" s="3" t="s">
         <v>72</v>
@@ -939,7 +939,7 @@
         <v>1</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>96</v>
+        <v>121</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>64</v>
@@ -951,13 +951,13 @@
         <v>43</v>
       </c>
       <c r="F3">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="G3" t="s">
         <v>41</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>110</v>
+        <v>123</v>
       </c>
       <c r="I3" s="1" t="s">
         <v>38</v>
@@ -972,7 +972,7 @@
         <v>49</v>
       </c>
       <c r="M3" s="3" t="s">
-        <v>111</v>
+        <v>124</v>
       </c>
       <c r="N3" s="3" t="s">
         <v>38</v>
@@ -987,7 +987,7 @@
         <v>50</v>
       </c>
       <c r="R3" s="3" t="s">
-        <v>112</v>
+        <v>87</v>
       </c>
       <c r="S3" s="3" t="s">
         <v>72</v>
@@ -1007,7 +1007,7 @@
         <v>0</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>101</v>
+        <v>86</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>64</v>
@@ -1025,7 +1025,7 @@
         <v>37</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="I4" s="1" t="s">
         <v>45</v>
@@ -1040,7 +1040,7 @@
         <v>41</v>
       </c>
       <c r="M4" s="3" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="N4" s="1" t="s">
         <v>45</v>
@@ -1055,7 +1055,7 @@
         <v>49</v>
       </c>
       <c r="R4" s="3" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="S4" s="1" t="s">
         <v>45</v>
@@ -1070,7 +1070,7 @@
         <v>50</v>
       </c>
       <c r="W4" s="3" t="s">
-        <v>105</v>
+        <v>82</v>
       </c>
       <c r="X4" s="1" t="s">
         <v>51</v>
@@ -1093,7 +1093,7 @@
         <v>0</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>64</v>
@@ -1111,7 +1111,7 @@
         <v>41</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>84</v>
+        <v>102</v>
       </c>
       <c r="I5" s="1" t="s">
         <v>45</v>
@@ -1126,7 +1126,7 @@
         <v>49</v>
       </c>
       <c r="M5" s="3" t="s">
-        <v>74</v>
+        <v>103</v>
       </c>
       <c r="N5" s="1" t="s">
         <v>45</v>
@@ -1141,7 +1141,7 @@
         <v>50</v>
       </c>
       <c r="R5" s="3" t="s">
-        <v>85</v>
+        <v>104</v>
       </c>
       <c r="S5" s="1" t="s">
         <v>51</v>
@@ -1163,7 +1163,7 @@
         <v>0</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>97</v>
+        <v>85</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>65</v>
@@ -1181,7 +1181,7 @@
         <v>37</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>93</v>
+        <v>109</v>
       </c>
       <c r="I6" s="1" t="s">
         <v>47</v>
@@ -1196,7 +1196,7 @@
         <v>41</v>
       </c>
       <c r="M6" s="3" t="s">
-        <v>94</v>
+        <v>110</v>
       </c>
       <c r="N6" s="1" t="s">
         <v>47</v>
@@ -1217,7 +1217,7 @@
         <v>0</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>91</v>
+        <v>83</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>65</v>
@@ -1235,7 +1235,7 @@
         <v>37</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>87</v>
+        <v>105</v>
       </c>
       <c r="I7" s="1" t="s">
         <v>45</v>
@@ -1250,7 +1250,7 @@
         <v>41</v>
       </c>
       <c r="M7" s="3" t="s">
-        <v>88</v>
+        <v>106</v>
       </c>
       <c r="N7" s="1" t="s">
         <v>45</v>
@@ -1265,7 +1265,7 @@
         <v>49</v>
       </c>
       <c r="R7" s="3" t="s">
-        <v>89</v>
+        <v>107</v>
       </c>
       <c r="S7" s="1" t="s">
         <v>45</v>
@@ -1280,7 +1280,7 @@
         <v>50</v>
       </c>
       <c r="W7" s="3" t="s">
-        <v>90</v>
+        <v>108</v>
       </c>
       <c r="X7" s="1" t="s">
         <v>51</v>
@@ -1315,7 +1315,7 @@
         <v>41</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>98</v>
+        <v>111</v>
       </c>
       <c r="I8" s="1" t="s">
         <v>58</v>
@@ -1330,7 +1330,7 @@
         <v>49</v>
       </c>
       <c r="M8" s="3" t="s">
-        <v>99</v>
+        <v>112</v>
       </c>
       <c r="N8" s="1" t="s">
         <v>58</v>
@@ -1345,7 +1345,7 @@
         <v>50</v>
       </c>
       <c r="R8" s="3" t="s">
-        <v>100</v>
+        <v>113</v>
       </c>
       <c r="S8" s="1" t="s">
         <v>51</v>
@@ -1366,7 +1366,7 @@
         <v>0</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>92</v>
+        <v>84</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>65</v>
@@ -1384,7 +1384,7 @@
         <v>50</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>86</v>
+        <v>114</v>
       </c>
       <c r="I9" s="1" t="s">
         <v>59</v>
@@ -1401,13 +1401,13 @@
         <v>0</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>79</v>
+        <v>117</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>65</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="E10" t="s">
         <v>54</v>
@@ -1419,16 +1419,16 @@
         <v>42</v>
       </c>
       <c r="H10" s="3" t="s">
-        <v>106</v>
+        <v>115</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="J10" s="1" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="K10" s="3" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="11" spans="1:36">
@@ -1436,7 +1436,7 @@
         <v>0</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>107</v>
+        <v>118</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>65</v>
@@ -1451,19 +1451,19 @@
         <v>2025</v>
       </c>
       <c r="G11" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="H11" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="I11" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="H11" s="3" t="s">
-        <v>108</v>
-      </c>
-      <c r="I11" s="3" t="s">
+      <c r="J11" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="J11" s="3" t="s">
+      <c r="K11" s="3" t="s">
         <v>77</v>
-      </c>
-      <c r="K11" s="3" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="12" spans="1:36">
@@ -1471,13 +1471,13 @@
         <v>0</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>124</v>
+        <v>98</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>120</v>
+        <v>95</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>121</v>
+        <v>96</v>
       </c>
       <c r="E12" t="s">
         <v>54</v>
@@ -1489,16 +1489,16 @@
         <v>50</v>
       </c>
       <c r="H12" s="3" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="I12" s="3" t="s">
         <v>58</v>
       </c>
       <c r="J12" s="3" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="K12" s="3" t="s">
-        <v>123</v>
+        <v>97</v>
       </c>
     </row>
     <row r="13" spans="1:36">
@@ -1506,7 +1506,7 @@
         <v>0</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>117</v>
+        <v>92</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>66</v>
@@ -1524,7 +1524,7 @@
         <v>41</v>
       </c>
       <c r="H13" s="3" t="s">
-        <v>118</v>
+        <v>93</v>
       </c>
       <c r="I13" s="1" t="s">
         <v>61</v>
@@ -1559,7 +1559,7 @@
         <v>49</v>
       </c>
       <c r="H14" s="3" t="s">
-        <v>119</v>
+        <v>94</v>
       </c>
       <c r="I14" s="1" t="s">
         <v>61</v>
@@ -1576,13 +1576,13 @@
         <v>0</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>113</v>
+        <v>88</v>
       </c>
       <c r="C15" s="2" t="s">
         <v>66</v>
       </c>
       <c r="D15" t="s">
-        <v>114</v>
+        <v>89</v>
       </c>
       <c r="E15" t="s">
         <v>54</v>
@@ -1591,10 +1591,10 @@
         <v>2025</v>
       </c>
       <c r="G15" t="s">
-        <v>116</v>
+        <v>91</v>
       </c>
       <c r="H15" s="3" t="s">
-        <v>115</v>
+        <v>90</v>
       </c>
       <c r="I15" s="1" t="s">
         <v>61</v>

</xml_diff>

<commit_message>
Se actualiza código, se agrega linea para utilizar la versión instalada de chrome: 06022026
</commit_message>
<xml_diff>
--- a/MazdaMX2/Dealers.xlsx
+++ b/MazdaMX2/Dealers.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mvelasc2\source\repos\MazdaMX2\MazdaMX2\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\manuelvelasco\source\repos\Mvelasco-git\MazdaMX2\MazdaMX2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{675549AD-CE16-4874-9755-C2AD9D21E7AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CEAEFF7-2978-4E88-B079-C73FF362942E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-118" yWindow="-118" windowWidth="25370" windowHeight="13667" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="22636" windowHeight="13546" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="2" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="242" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="128">
   <si>
     <t>VERIFICAR</t>
   </si>
@@ -235,9 +235,6 @@
     <t>cx-5-flydown-perfil-v1</t>
   </si>
   <si>
-    <t>carro-mazda-mx-5-gris-v1</t>
-  </si>
-  <si>
     <t>141</t>
   </si>
   <si>
@@ -271,15 +268,6 @@
     <t>552,900</t>
   </si>
   <si>
-    <t>mazda-cx-30-flydown-perfil-v2</t>
-  </si>
-  <si>
-    <t>mazda-cx-50-flydown-v2</t>
-  </si>
-  <si>
-    <t>mazda-mexico-cx-3-flydown-perfil-v1</t>
-  </si>
-  <si>
     <t>mazda3-sedan-flydown-perfil-v2</t>
   </si>
   <si>
@@ -298,15 +286,6 @@
     <t>35° Aniversario</t>
   </si>
   <si>
-    <t>mx-5-carro-rojo-deportivo-inclinado-v1-1</t>
-  </si>
-  <si>
-    <t>529,900</t>
-  </si>
-  <si>
-    <t>629,900</t>
-  </si>
-  <si>
     <t>PICKUPS</t>
   </si>
   <si>
@@ -337,24 +316,6 @@
     <t>568,900</t>
   </si>
   <si>
-    <t>441,900</t>
-  </si>
-  <si>
-    <t>471,900</t>
-  </si>
-  <si>
-    <t>517,900</t>
-  </si>
-  <si>
-    <t>557,900</t>
-  </si>
-  <si>
-    <t>391,900</t>
-  </si>
-  <si>
-    <t>421,900</t>
-  </si>
-  <si>
     <t>551,900</t>
   </si>
   <si>
@@ -364,24 +325,9 @@
     <t>681,900</t>
   </si>
   <si>
-    <t>818,900</t>
-  </si>
-  <si>
-    <t>961,000</t>
-  </si>
-  <si>
-    <t>1,061,000</t>
-  </si>
-  <si>
-    <t>mazda-cx-70-racks-flydown-inclinado-v1</t>
-  </si>
-  <si>
     <t>mazda-cx-90-flydown-rojo-artesano-inclinado-v1</t>
   </si>
   <si>
-    <t>799,900</t>
-  </si>
-  <si>
     <t>mazda2-sedan-rojo-auto-perfil-v1</t>
   </si>
   <si>
@@ -395,6 +341,69 @@
   </si>
   <si>
     <t>371,900</t>
+  </si>
+  <si>
+    <t>Signature MHEV (Asientos Capitán)</t>
+  </si>
+  <si>
+    <t>502,900</t>
+  </si>
+  <si>
+    <t>153</t>
+  </si>
+  <si>
+    <t>Carbon Edition MHEV</t>
+  </si>
+  <si>
+    <t>mazda-cx70-flydown-perfil-v1</t>
+  </si>
+  <si>
+    <t>mazda-mx-5-auto-rojo-deportivo-perfil-v1</t>
+  </si>
+  <si>
+    <t>auto-mazda-mx-5-rf-gris-titanio-perfil-v1</t>
+  </si>
+  <si>
+    <t>mazda-cx-3-flydown-perfil-v1</t>
+  </si>
+  <si>
+    <t>mazda-cx30-camioneta-roja-flydown-perfil-v1</t>
+  </si>
+  <si>
+    <t>mazda-cx50-suv-verde-flydown-v1</t>
+  </si>
+  <si>
+    <t>837,900</t>
+  </si>
+  <si>
+    <t>996,900</t>
+  </si>
+  <si>
+    <t>1,011,900</t>
+  </si>
+  <si>
+    <t>829,900</t>
+  </si>
+  <si>
+    <t>546,900</t>
+  </si>
+  <si>
+    <t>646,900</t>
+  </si>
+  <si>
+    <t>432,900</t>
+  </si>
+  <si>
+    <t>451,900</t>
+  </si>
+  <si>
+    <t>481,900</t>
+  </si>
+  <si>
+    <t>525,900</t>
+  </si>
+  <si>
+    <t>577,900</t>
   </si>
 </sst>
 </file>
@@ -718,30 +727,30 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AJ15"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.77734375" defaultRowHeight="15.75"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.75" defaultRowHeight="15.75"/>
   <cols>
-    <col min="1" max="1" width="12.77734375" customWidth="1"/>
-    <col min="2" max="2" width="30.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.77734375" customWidth="1"/>
-    <col min="4" max="4" width="12.109375" customWidth="1"/>
-    <col min="5" max="5" width="10.77734375" customWidth="1"/>
+    <col min="1" max="1" width="12.75" customWidth="1"/>
+    <col min="2" max="2" width="30.3125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.75" customWidth="1"/>
+    <col min="4" max="4" width="12.125" customWidth="1"/>
+    <col min="5" max="5" width="10.75" customWidth="1"/>
     <col min="6" max="6" width="8" customWidth="1"/>
-    <col min="7" max="7" width="13.21875" customWidth="1"/>
+    <col min="7" max="7" width="13.25" customWidth="1"/>
     <col min="8" max="8" width="9" style="1"/>
     <col min="9" max="9" width="4" style="1" customWidth="1"/>
-    <col min="10" max="10" width="8.77734375" style="1" customWidth="1"/>
-    <col min="11" max="11" width="9.21875" style="1" customWidth="1"/>
-    <col min="12" max="12" width="13.21875" customWidth="1"/>
+    <col min="10" max="10" width="8.75" style="1" customWidth="1"/>
+    <col min="11" max="11" width="9.25" style="1" customWidth="1"/>
+    <col min="12" max="12" width="13.25" customWidth="1"/>
     <col min="13" max="13" width="9" style="1"/>
-    <col min="14" max="15" width="8.77734375" style="1"/>
-    <col min="16" max="16" width="9.21875" style="1" customWidth="1"/>
-    <col min="17" max="17" width="13.77734375" customWidth="1"/>
+    <col min="14" max="15" width="8.75" style="1"/>
+    <col min="16" max="16" width="9.25" style="1" customWidth="1"/>
+    <col min="17" max="17" width="13.75" customWidth="1"/>
     <col min="18" max="18" width="9" style="1"/>
-    <col min="19" max="21" width="8.77734375" style="1"/>
-    <col min="22" max="22" width="13.88671875" customWidth="1"/>
-    <col min="25" max="25" width="8.77734375" customWidth="1"/>
-    <col min="27" max="27" width="10.109375" customWidth="1"/>
-    <col min="32" max="32" width="13.88671875" customWidth="1"/>
+    <col min="19" max="21" width="8.75" style="1"/>
+    <col min="22" max="22" width="13.875" customWidth="1"/>
+    <col min="25" max="25" width="8.75" customWidth="1"/>
+    <col min="27" max="27" width="10.125" customWidth="1"/>
+    <col min="32" max="32" width="13.875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:36">
@@ -859,7 +868,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>120</v>
+        <v>102</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>64</v>
@@ -877,7 +886,7 @@
         <v>37</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>122</v>
+        <v>104</v>
       </c>
       <c r="I2" s="1" t="s">
         <v>38</v>
@@ -892,7 +901,7 @@
         <v>41</v>
       </c>
       <c r="M2" s="3" t="s">
-        <v>123</v>
+        <v>105</v>
       </c>
       <c r="N2" s="1" t="s">
         <v>38</v>
@@ -907,7 +916,7 @@
         <v>49</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>124</v>
+        <v>106</v>
       </c>
       <c r="S2" s="3" t="s">
         <v>38</v>
@@ -922,13 +931,13 @@
         <v>50</v>
       </c>
       <c r="W2" s="3" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="X2" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="Y2" s="3" t="s">
         <v>72</v>
-      </c>
-      <c r="Y2" s="3" t="s">
-        <v>73</v>
       </c>
       <c r="Z2" s="3" t="s">
         <v>48</v>
@@ -939,7 +948,7 @@
         <v>1</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>121</v>
+        <v>103</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>64</v>
@@ -957,7 +966,7 @@
         <v>41</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>123</v>
+        <v>105</v>
       </c>
       <c r="I3" s="1" t="s">
         <v>38</v>
@@ -972,7 +981,7 @@
         <v>49</v>
       </c>
       <c r="M3" s="3" t="s">
-        <v>124</v>
+        <v>106</v>
       </c>
       <c r="N3" s="3" t="s">
         <v>38</v>
@@ -987,13 +996,13 @@
         <v>50</v>
       </c>
       <c r="R3" s="3" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="S3" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="T3" s="3" t="s">
         <v>72</v>
-      </c>
-      <c r="T3" s="3" t="s">
-        <v>73</v>
       </c>
       <c r="U3" s="3" t="s">
         <v>48</v>
@@ -1004,10 +1013,10 @@
     </row>
     <row r="4" spans="1:36">
       <c r="A4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>64</v>
@@ -1019,13 +1028,13 @@
         <v>36</v>
       </c>
       <c r="F4">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="G4" t="s">
         <v>37</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>99</v>
+        <v>92</v>
       </c>
       <c r="I4" s="1" t="s">
         <v>45</v>
@@ -1040,7 +1049,7 @@
         <v>41</v>
       </c>
       <c r="M4" s="3" t="s">
-        <v>100</v>
+        <v>93</v>
       </c>
       <c r="N4" s="1" t="s">
         <v>45</v>
@@ -1055,7 +1064,7 @@
         <v>49</v>
       </c>
       <c r="R4" s="3" t="s">
-        <v>101</v>
+        <v>94</v>
       </c>
       <c r="S4" s="1" t="s">
         <v>45</v>
@@ -1067,33 +1076,45 @@
         <v>46</v>
       </c>
       <c r="V4" t="s">
+        <v>42</v>
+      </c>
+      <c r="W4" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="X4" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="Y4" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="Z4" t="s">
+        <v>48</v>
+      </c>
+      <c r="AA4" t="s">
         <v>50</v>
       </c>
-      <c r="W4" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="X4" s="1" t="s">
+      <c r="AB4" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="AC4" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="Y4" s="1" t="s">
+      <c r="AD4" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="Z4" t="s">
+      <c r="AE4" t="s">
         <v>46</v>
       </c>
-      <c r="AB4" s="3"/>
-      <c r="AC4" s="1"/>
-      <c r="AD4" s="1"/>
       <c r="AG4" s="1"/>
       <c r="AH4" s="1"/>
       <c r="AI4" s="1"/>
     </row>
     <row r="5" spans="1:36">
       <c r="A5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>64</v>
@@ -1105,13 +1126,13 @@
         <v>43</v>
       </c>
       <c r="F5">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="G5" t="s">
         <v>41</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>102</v>
+        <v>95</v>
       </c>
       <c r="I5" s="1" t="s">
         <v>45</v>
@@ -1126,7 +1147,7 @@
         <v>49</v>
       </c>
       <c r="M5" s="3" t="s">
-        <v>103</v>
+        <v>96</v>
       </c>
       <c r="N5" s="1" t="s">
         <v>45</v>
@@ -1141,7 +1162,7 @@
         <v>50</v>
       </c>
       <c r="R5" s="3" t="s">
-        <v>104</v>
+        <v>97</v>
       </c>
       <c r="S5" s="1" t="s">
         <v>51</v>
@@ -1160,10 +1181,10 @@
     </row>
     <row r="6" spans="1:36">
       <c r="A6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>85</v>
+        <v>114</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>65</v>
@@ -1175,13 +1196,13 @@
         <v>54</v>
       </c>
       <c r="F6">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="G6" t="s">
         <v>37</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>109</v>
+        <v>92</v>
       </c>
       <c r="I6" s="1" t="s">
         <v>47</v>
@@ -1196,7 +1217,7 @@
         <v>41</v>
       </c>
       <c r="M6" s="3" t="s">
-        <v>110</v>
+        <v>123</v>
       </c>
       <c r="N6" s="1" t="s">
         <v>47</v>
@@ -1214,10 +1235,10 @@
     </row>
     <row r="7" spans="1:36">
       <c r="A7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>83</v>
+        <v>115</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>65</v>
@@ -1229,13 +1250,13 @@
         <v>54</v>
       </c>
       <c r="F7">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="G7" t="s">
         <v>37</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>105</v>
+        <v>124</v>
       </c>
       <c r="I7" s="1" t="s">
         <v>45</v>
@@ -1250,7 +1271,7 @@
         <v>41</v>
       </c>
       <c r="M7" s="3" t="s">
-        <v>106</v>
+        <v>125</v>
       </c>
       <c r="N7" s="1" t="s">
         <v>45</v>
@@ -1265,7 +1286,7 @@
         <v>49</v>
       </c>
       <c r="R7" s="3" t="s">
-        <v>107</v>
+        <v>126</v>
       </c>
       <c r="S7" s="1" t="s">
         <v>45</v>
@@ -1280,7 +1301,7 @@
         <v>50</v>
       </c>
       <c r="W7" s="3" t="s">
-        <v>108</v>
+        <v>127</v>
       </c>
       <c r="X7" s="1" t="s">
         <v>51</v>
@@ -1315,7 +1336,7 @@
         <v>41</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>111</v>
+        <v>98</v>
       </c>
       <c r="I8" s="1" t="s">
         <v>58</v>
@@ -1330,7 +1351,7 @@
         <v>49</v>
       </c>
       <c r="M8" s="3" t="s">
-        <v>112</v>
+        <v>99</v>
       </c>
       <c r="N8" s="1" t="s">
         <v>58</v>
@@ -1345,7 +1366,7 @@
         <v>50</v>
       </c>
       <c r="R8" s="3" t="s">
-        <v>113</v>
+        <v>100</v>
       </c>
       <c r="S8" s="1" t="s">
         <v>51</v>
@@ -1366,7 +1387,7 @@
         <v>0</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>84</v>
+        <v>116</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>65</v>
@@ -1378,13 +1399,13 @@
         <v>54</v>
       </c>
       <c r="F9">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="G9" s="2" t="s">
         <v>50</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="I9" s="1" t="s">
         <v>59</v>
@@ -1401,34 +1422,34 @@
         <v>0</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>65</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="E10" t="s">
         <v>54</v>
       </c>
       <c r="F10">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="G10" t="s">
-        <v>42</v>
+        <v>110</v>
       </c>
       <c r="H10" s="3" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="I10" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="J10" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="J10" s="1" t="s">
-        <v>81</v>
-      </c>
       <c r="K10" s="3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="11" spans="1:36">
@@ -1436,7 +1457,7 @@
         <v>0</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>118</v>
+        <v>101</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>65</v>
@@ -1448,22 +1469,37 @@
         <v>54</v>
       </c>
       <c r="F11">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="G11" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="H11" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="I11" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="H11" s="3" t="s">
-        <v>116</v>
-      </c>
-      <c r="I11" s="3" t="s">
+      <c r="J11" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="J11" s="3" t="s">
+      <c r="K11" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="K11" s="3" t="s">
-        <v>77</v>
+      <c r="L11" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="M11" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="N11" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="O11" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="P11" s="3" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="12" spans="1:36">
@@ -1471,13 +1507,13 @@
         <v>0</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>98</v>
+        <v>91</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>95</v>
+        <v>88</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>96</v>
+        <v>89</v>
       </c>
       <c r="E12" t="s">
         <v>54</v>
@@ -1489,16 +1525,16 @@
         <v>50</v>
       </c>
       <c r="H12" s="3" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="I12" s="3" t="s">
         <v>58</v>
       </c>
       <c r="J12" s="3" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="K12" s="3" t="s">
-        <v>97</v>
+        <v>90</v>
       </c>
     </row>
     <row r="13" spans="1:36">
@@ -1506,7 +1542,7 @@
         <v>0</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>92</v>
+        <v>112</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>66</v>
@@ -1518,13 +1554,13 @@
         <v>54</v>
       </c>
       <c r="F13">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="G13" t="s">
         <v>41</v>
       </c>
       <c r="H13" s="3" t="s">
-        <v>93</v>
+        <v>121</v>
       </c>
       <c r="I13" s="1" t="s">
         <v>61</v>
@@ -1541,7 +1577,7 @@
         <v>0</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>71</v>
+        <v>113</v>
       </c>
       <c r="C14" s="2" t="s">
         <v>66</v>
@@ -1553,13 +1589,13 @@
         <v>54</v>
       </c>
       <c r="F14">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="G14" t="s">
         <v>49</v>
       </c>
       <c r="H14" s="3" t="s">
-        <v>94</v>
+        <v>122</v>
       </c>
       <c r="I14" s="1" t="s">
         <v>61</v>
@@ -1576,13 +1612,13 @@
         <v>0</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="C15" s="2" t="s">
         <v>66</v>
       </c>
       <c r="D15" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="E15" t="s">
         <v>54</v>
@@ -1591,10 +1627,10 @@
         <v>2025</v>
       </c>
       <c r="G15" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="H15" s="3" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="I15" s="1" t="s">
         <v>61</v>

</xml_diff>

<commit_message>
Se sube nuevo código mejorando la lectura del archivo excel solo una vez en la ejecución.
</commit_message>
<xml_diff>
--- a/MazdaMX2/Dealers.xlsx
+++ b/MazdaMX2/Dealers.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\manuelvelasco\source\repos\Mvelasco-git\MazdaMX2\MazdaMX2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CEAEFF7-2978-4E88-B079-C73FF362942E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{475496F1-4F42-46F7-96D5-998969CF7D01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="22636" windowHeight="13546" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15675" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="2" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="128">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="271" uniqueCount="133">
   <si>
     <t>VERIFICAR</t>
   </si>
@@ -382,9 +382,6 @@
     <t>1,011,900</t>
   </si>
   <si>
-    <t>829,900</t>
-  </si>
-  <si>
     <t>546,900</t>
   </si>
   <si>
@@ -404,6 +401,24 @@
   </si>
   <si>
     <t>577,900</t>
+  </si>
+  <si>
+    <t>723,900</t>
+  </si>
+  <si>
+    <t>mazda-cx5-2026-flydown-perfil-v1</t>
+  </si>
+  <si>
+    <t>599,900</t>
+  </si>
+  <si>
+    <t>177</t>
+  </si>
+  <si>
+    <t>659,900</t>
+  </si>
+  <si>
+    <t>719,900</t>
   </si>
 </sst>
 </file>
@@ -726,7 +741,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AJ15"/>
+  <dimension ref="A1:AJ16"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.75" defaultRowHeight="15.75"/>
   <cols>
     <col min="1" max="1" width="12.75" customWidth="1"/>
@@ -865,7 +880,7 @@
     </row>
     <row r="2" spans="1:36">
       <c r="A2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>102</v>
@@ -945,7 +960,7 @@
     </row>
     <row r="3" spans="1:36">
       <c r="A3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>103</v>
@@ -1013,7 +1028,7 @@
     </row>
     <row r="4" spans="1:36">
       <c r="A4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>82</v>
@@ -1111,7 +1126,7 @@
     </row>
     <row r="5" spans="1:36">
       <c r="A5" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>78</v>
@@ -1181,7 +1196,7 @@
     </row>
     <row r="6" spans="1:36">
       <c r="A6" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>114</v>
@@ -1217,7 +1232,7 @@
         <v>41</v>
       </c>
       <c r="M6" s="3" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="N6" s="1" t="s">
         <v>47</v>
@@ -1235,7 +1250,7 @@
     </row>
     <row r="7" spans="1:36">
       <c r="A7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>115</v>
@@ -1256,7 +1271,7 @@
         <v>37</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="I7" s="1" t="s">
         <v>45</v>
@@ -1271,7 +1286,7 @@
         <v>41</v>
       </c>
       <c r="M7" s="3" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="N7" s="1" t="s">
         <v>45</v>
@@ -1286,7 +1301,7 @@
         <v>49</v>
       </c>
       <c r="R7" s="3" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="S7" s="1" t="s">
         <v>45</v>
@@ -1301,7 +1316,7 @@
         <v>50</v>
       </c>
       <c r="W7" s="3" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="X7" s="1" t="s">
         <v>51</v>
@@ -1384,16 +1399,16 @@
     </row>
     <row r="9" spans="1:36">
       <c r="A9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>116</v>
+        <v>128</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>65</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="E9" t="s">
         <v>54</v>
@@ -1401,34 +1416,68 @@
       <c r="F9">
         <v>2026</v>
       </c>
-      <c r="G9" s="2" t="s">
-        <v>50</v>
+      <c r="G9" t="s">
+        <v>41</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>117</v>
+        <v>129</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>59</v>
+        <v>130</v>
       </c>
       <c r="J9" s="1" t="s">
-        <v>52</v>
+        <v>130</v>
       </c>
       <c r="K9" s="1" t="s">
         <v>46</v>
       </c>
+      <c r="L9" t="s">
+        <v>49</v>
+      </c>
+      <c r="M9" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="N9" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="O9" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="P9" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="Q9" t="s">
+        <v>50</v>
+      </c>
+      <c r="R9" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="S9" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="T9" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="U9" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="W9" s="1"/>
+      <c r="X9" s="1"/>
+      <c r="Y9" s="1"/>
+      <c r="Z9" s="1"/>
     </row>
     <row r="10" spans="1:36">
       <c r="A10" t="b">
         <v>0</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>65</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>77</v>
+        <v>67</v>
       </c>
       <c r="E10" t="s">
         <v>54</v>
@@ -1436,20 +1485,20 @@
       <c r="F10">
         <v>2026</v>
       </c>
-      <c r="G10" t="s">
-        <v>110</v>
+      <c r="G10" s="2" t="s">
+        <v>50</v>
       </c>
       <c r="H10" s="3" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>79</v>
+        <v>59</v>
       </c>
       <c r="J10" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="K10" s="3" t="s">
-        <v>76</v>
+        <v>52</v>
+      </c>
+      <c r="K10" s="1" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="11" spans="1:36">
@@ -1457,13 +1506,13 @@
         <v>0</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>65</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>68</v>
+        <v>77</v>
       </c>
       <c r="E11" t="s">
         <v>54</v>
@@ -1471,34 +1520,19 @@
       <c r="F11">
         <v>2026</v>
       </c>
-      <c r="G11" s="2" t="s">
-        <v>73</v>
+      <c r="G11" t="s">
+        <v>110</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="I11" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="J11" s="3" t="s">
-        <v>75</v>
+        <v>118</v>
+      </c>
+      <c r="I11" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="J11" s="1" t="s">
+        <v>80</v>
       </c>
       <c r="K11" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="L11" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="M11" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="N11" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="O11" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="P11" s="3" t="s">
         <v>76</v>
       </c>
     </row>
@@ -1507,34 +1541,49 @@
         <v>0</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>91</v>
+        <v>101</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>88</v>
+        <v>65</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>89</v>
+        <v>68</v>
       </c>
       <c r="E12" t="s">
         <v>54</v>
       </c>
       <c r="F12">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>50</v>
+        <v>73</v>
       </c>
       <c r="H12" s="3" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="I12" s="3" t="s">
-        <v>58</v>
+        <v>74</v>
       </c>
       <c r="J12" s="3" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="K12" s="3" t="s">
-        <v>90</v>
+        <v>76</v>
+      </c>
+      <c r="L12" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="M12" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="N12" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="O12" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="P12" s="3" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="13" spans="1:36">
@@ -1542,34 +1591,34 @@
         <v>0</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>112</v>
+        <v>91</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="D13" t="s">
-        <v>60</v>
+        <v>88</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>89</v>
       </c>
       <c r="E13" t="s">
         <v>54</v>
       </c>
       <c r="F13">
-        <v>2026</v>
-      </c>
-      <c r="G13" t="s">
-        <v>41</v>
+        <v>2025</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>50</v>
       </c>
       <c r="H13" s="3" t="s">
-        <v>121</v>
-      </c>
-      <c r="I13" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="J13" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="K13" s="1" t="s">
-        <v>48</v>
+        <v>127</v>
+      </c>
+      <c r="I13" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="J13" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="K13" s="3" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="14" spans="1:36">
@@ -1577,13 +1626,13 @@
         <v>0</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C14" s="2" t="s">
         <v>66</v>
       </c>
       <c r="D14" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="E14" t="s">
         <v>54</v>
@@ -1592,10 +1641,10 @@
         <v>2026</v>
       </c>
       <c r="G14" t="s">
-        <v>49</v>
+        <v>41</v>
       </c>
       <c r="H14" s="3" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="I14" s="1" t="s">
         <v>61</v>
@@ -1612,25 +1661,25 @@
         <v>0</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>84</v>
+        <v>113</v>
       </c>
       <c r="C15" s="2" t="s">
         <v>66</v>
       </c>
       <c r="D15" t="s">
-        <v>85</v>
+        <v>63</v>
       </c>
       <c r="E15" t="s">
         <v>54</v>
       </c>
       <c r="F15">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="G15" t="s">
-        <v>87</v>
+        <v>49</v>
       </c>
       <c r="H15" s="3" t="s">
-        <v>86</v>
+        <v>121</v>
       </c>
       <c r="I15" s="1" t="s">
         <v>61</v>
@@ -1639,6 +1688,41 @@
         <v>62</v>
       </c>
       <c r="K15" s="1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="16" spans="1:36">
+      <c r="A16" t="b">
+        <v>0</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="D16" t="s">
+        <v>85</v>
+      </c>
+      <c r="E16" t="s">
+        <v>54</v>
+      </c>
+      <c r="F16">
+        <v>2025</v>
+      </c>
+      <c r="G16" t="s">
+        <v>87</v>
+      </c>
+      <c r="H16" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="I16" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="J16" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="K16" s="1" t="s">
         <v>48</v>
       </c>
     </row>

</xml_diff>